<commit_message>
Fix site coordinates and Excel parser numeric-value bug
- Update all 10 site coordinates to verified HQ locations from public sources
- Reagan Test Site moved from Roi-Namur radar island to Kwajalein Island HQ
- Other sites adjusted by 0-2km to align with published Wikipedia HQ coordinates

Parser fix: formula-injection prevention was prepending a single quote to any
string starting with "-", which corrupted negative numeric values (longitudes)
into NaN -> 0. Sanitize now bypasses numeric/boolean values directly and only
treats a leading "-" as suspicious if the string is not parseable as a number.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/us_missile_range_data.xlsx
+++ b/data/us_missile_range_data.xlsx
@@ -2206,10 +2206,10 @@
         <v>27</v>
       </c>
       <c r="H2">
-        <v>32.3829</v>
+        <v>32.3831</v>
       </c>
       <c r="I2">
-        <v>-106.4783</v>
+        <v>-106.4781</v>
       </c>
       <c r="J2" t="s">
         <v>28</v>
@@ -2268,10 +2268,10 @@
         <v>42</v>
       </c>
       <c r="H3">
-        <v>34.742</v>
+        <v>34.7333</v>
       </c>
       <c r="I3">
-        <v>-120.5724</v>
+        <v>-120.5667</v>
       </c>
       <c r="J3" t="s">
         <v>28</v>
@@ -2392,10 +2392,10 @@
         <v>62</v>
       </c>
       <c r="H5">
-        <v>9.3948</v>
+        <v>8.7181</v>
       </c>
       <c r="I5">
-        <v>167.471</v>
+        <v>167.7328</v>
       </c>
       <c r="J5" t="s">
         <v>28</v>
@@ -2451,10 +2451,10 @@
         <v>70</v>
       </c>
       <c r="H6">
-        <v>22.0227</v>
+        <v>22.0394</v>
       </c>
       <c r="I6">
-        <v>-159.785</v>
+        <v>-159.7853</v>
       </c>
       <c r="J6" t="s">
         <v>28</v>
@@ -2513,10 +2513,10 @@
         <v>80</v>
       </c>
       <c r="H7">
-        <v>37.9402</v>
+        <v>37.94</v>
       </c>
       <c r="I7">
-        <v>-75.4664</v>
+        <v>-75.4661</v>
       </c>
       <c r="J7" t="s">
         <v>28</v>
@@ -2572,10 +2572,10 @@
         <v>52</v>
       </c>
       <c r="H8">
-        <v>30.4727</v>
+        <v>30.475</v>
       </c>
       <c r="I8">
-        <v>-86.5264</v>
+        <v>-86.5256</v>
       </c>
       <c r="J8" t="s">
         <v>28</v>
@@ -2631,7 +2631,7 @@
         <v>98</v>
       </c>
       <c r="H9">
-        <v>65.1296</v>
+        <v>65.1211</v>
       </c>
       <c r="I9">
         <v>-147.47</v>
@@ -2690,10 +2690,10 @@
         <v>107</v>
       </c>
       <c r="H10">
-        <v>37.7988</v>
+        <v>37.7981</v>
       </c>
       <c r="I10">
-        <v>-116.7809</v>
+        <v>-116.7806</v>
       </c>
       <c r="J10" t="s">
         <v>28</v>
@@ -2749,10 +2749,10 @@
         <v>98</v>
       </c>
       <c r="H11">
-        <v>57.4358</v>
+        <v>57.4333</v>
       </c>
       <c r="I11">
-        <v>-152.3378</v>
+        <v>-152.3333</v>
       </c>
       <c r="J11" t="s">
         <v>28</v>

</xml_diff>